<commit_message>
Docs: upload column (A / E) for Part List and Mapping upload templates
- XD01 / XD02 UISS: flag_add_edit renamed to upload; XD03 UISS: new upload column, check 8, sample E9
- apply_2710.py registered in build_all_v2.sh; upload modal screenshots retaken
- md X1-X4, XD01-XD03 and UR summary updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/XD01-XD15_UR_Business_Logic_Summary.xlsx
+++ b/deliverables/function_list_v2/XD01-XD15_UR_Business_Logic_Summary.xlsx
@@ -886,7 +886,7 @@
       <c r="H6" s="4" t="inlineStr">
         <is>
           <t>1. All-or-nothing: 1 error = seluruh file ditolak.
-2. Flag A = part baru (Candidate), flag E = ubah; baris tanpa perubahan di-skip.
+2. Kolom upload: A = part baru (Candidate), E = ubah; baris tanpa perubahan di-skip.
 3. Max Case/Day tidak boleh &lt; total mapping.
 4. Result report + sheet Re-upload.</t>
         </is>
@@ -949,8 +949,9 @@
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>1. All-or-nothing.
-2. Part harus Active; destinasi ada di master H0125; 1 destinasi sekali per part.
-3. Total case_day per part ≤ Max Case/Day.
+2. Kolom upload A (destinasi baru) / E (sudah di-mapping).
+3. Part harus Active; destinasi ada di master H0125; 1 destinasi sekali per part.
+4. Total case_day per part ≤ Max Case/Day.
 4. Part berubah → replace seluruh mapping part + No Sync.</t>
         </is>
       </c>
@@ -2289,7 +2290,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>User Procurement upload file Excel (sheet "Upload") untuk Add (flag A) dan Edit (flag E) part.</t>
+          <t>User Procurement upload file Excel (sheet "Upload") untuk Add (upload = A) dan Edit (upload = E) part.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr"/>
@@ -2353,7 +2354,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Part ada di master; flag A belum terdaftar / flag E sudah terdaftar; tidak duplikat di file; min_mad bulat ≥ 0, pcs_case &amp; max_case_day bulat &gt; 0; status sesuai aturan (A kosong, E tidak boleh menjadi Candidate); Effective Start Date wajib selama Candidate dan ≥ hari ini; Max Case/Day ≥ total mapping.</t>
+          <t>upload = A atau E; part ada di master; A belum terdaftar / E sudah terdaftar; tidak duplikat di file; min_mad bulat ≥ 0, pcs_case &amp; max_case_day bulat &gt; 0; status sesuai aturan (A kosong, E tidak boleh menjadi Candidate); Effective Start Date wajib selama Candidate dan ≥ hari ini; Max Case/Day ≥ total mapping.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
@@ -2421,7 +2422,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Flag A insert status Candidate; flag E update kolom yang berubah (baris tanpa perubahan di-skip). Part tersimpan → SYNC_STATUS 0, LAST_SOURCE UPLOAD, history.</t>
+          <t>upload A insert status Candidate; upload E update kolom yang berubah (baris tanpa perubahan di-skip). Part tersimpan → SYNC_STATUS 0, LAST_SOURCE UPLOAD, history.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr"/>
@@ -2525,7 +2526,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Cek file sama dengan XD02 (4 kolom). Part ada dan Active; destinasi ada di TB_M_H0125_DESTINATION; destinasi tidak duplikat per part; case_day bulat &gt; 0; total per part ≤ Max Case/Day. Baris placeholder kosong di-skip.</t>
+          <t>Cek file sama dengan XD02 (5 kolom). Kolom upload: A = destinasi baru untuk part, E = destinasi yang sudah di-mapping (Export mengisi E, A untuk placeholder). Part ada dan Active; destinasi ada di TB_M_H0125_DESTINATION; destinasi tidak duplikat per part; case_day bulat &gt; 0; total per part ≤ Max Case/Day. Baris placeholder kosong di-skip.</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">

</xml_diff>

<commit_message>
XD01: remove incomplete-mapping counter from Part List; show mapped Case/Day in Edit (FB-024, FB-025)
- Prototype: Part List header shows 'N parts' only; Edit part data shows 'Mapped Case/Day (current period): n'
- UISS XD01 (apply_2810.py in build_all_v2.sh): objective, Registered parts counter, Incomplete mapping marker removed,
  new item Mapped Case/Day, Operation 5.3 / 5.5; 14 Part List screenshots retaken (part_list_shots.mjs)
- UR XD01 regenerated (FR-06 replaced), UR summary and prepare_code Markdown updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/XD01-XD15_UR_Business_Logic_Summary.xlsx
+++ b/deliverables/function_list_v2/XD01-XD15_UR_Business_Logic_Summary.xlsx
@@ -1862,17 +1862,13 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Filter Part No, Status (All / Candidate / Active / Inactive), Sort; diterapkan saat [Search]. 25/50/100 baris per halaman. Counter "N parts · M incomplete mappings".</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Incomplete mapping = part tanpa destinasi atau total Case/Day ≠ Max Case/Day (bar biru).</t>
-        </is>
-      </c>
+          <t>Filter Part No, Status (All / Candidate / Active / Inactive), Sort; diterapkan saat [Search]. 25/50/100 baris per halaman. Counter "N parts". Kelengkapan mapping dipantau D/S di tab Mapping per Destination (FB-024).</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>TB_M_PART_CANDIDATE, TB_M_PART_CANDIDATE_DEST</t>
+          <t>TB_M_PART_CANDIDATE</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2006,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Max Case/Day tidak boleh lebih kecil dari total Case/Day yang sudah di-mapping periode berjalan (MSG14, Save disabled). Kurangi mapping dulu.</t>
+          <t>Max Case/Day tidak boleh lebih kecil dari total Case/Day yang sudah di-mapping periode berjalan (MSG14, Save disabled). Modal Edit menampilkan "Mapped Case/Day (current period)" sebagai batas bawah (FB-025). Kurangi mapping dulu.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr"/>

</xml_diff>